<commit_message>
feat(calculators): implements method 1 and 2 for ch 3.1 beef feedlot enteric methane
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/3.1-beef-feedlot-enteric.xlsx
+++ b/packages/calculators/src/modules/test/3.1-beef-feedlot-enteric.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5456112D-1680-6E4C-B187-C427BCCB6600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE27BA62-0787-A345-8DC5-77A675A07915}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51720" yWindow="17760" windowWidth="26840" windowHeight="15680" xr2:uid="{983596DC-3B3D-3549-9B15-A60291DF034B}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="39">
   <si>
     <t>Nj</t>
   </si>
@@ -252,6 +252,12 @@
   </si>
   <si>
     <t>Baseline</t>
+  </si>
+  <si>
+    <t>Boundary durations</t>
+  </si>
+  <si>
+    <t>Empty groups</t>
   </si>
 </sst>
 </file>
@@ -650,7 +656,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3B5E9308-1946-8F47-9834-B86881D77B59}">
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:V33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.2">
@@ -854,15 +860,15 @@
         <v>0-80 days</v>
       </c>
       <c r="F11">
-        <f>VLOOKUP(E11, S5:V7, 2, FALSE)</f>
+        <f>VLOOKUP(E11, $S$5:$V$7, 2, FALSE)</f>
         <v>10.4</v>
       </c>
       <c r="G11">
-        <f>VLOOKUP(E11, S5:V7, 3, FALSE)</f>
+        <f>VLOOKUP(E11, $S$5:$V$7, 3, FALSE)</f>
         <v>22</v>
       </c>
       <c r="H11">
-        <f>VLOOKUP(E11, S5:V7, 4, FALSE)</f>
+        <f>VLOOKUP(E11, $S$5:$V$7, 4, FALSE)</f>
         <v>4.8</v>
       </c>
       <c r="I11">
@@ -901,15 +907,15 @@
         <v>81-200 days</v>
       </c>
       <c r="F12">
-        <f t="shared" ref="F12:F13" si="0">VLOOKUP(E12, S6:V8, 2, FALSE)</f>
+        <f t="shared" ref="F12:F13" si="0">VLOOKUP(E12, $S$5:$V$7, 2, FALSE)</f>
         <v>10.8</v>
       </c>
       <c r="G12">
-        <f t="shared" ref="G12:G13" si="1">VLOOKUP(E12, S6:V8, 3, FALSE)</f>
+        <f t="shared" ref="G12:G13" si="1">VLOOKUP(E12, $S$5:$V$7, 3, FALSE)</f>
         <v>22</v>
       </c>
       <c r="H12">
-        <f t="shared" ref="H12:H13" si="2">VLOOKUP(E12, S6:V8, 4, FALSE)</f>
+        <f t="shared" ref="H12:H13" si="2">VLOOKUP(E12, $S$5:$V$7, 4, FALSE)</f>
         <v>5</v>
       </c>
       <c r="I12">
@@ -954,6 +960,360 @@
       <c r="J13">
         <f t="shared" si="4"/>
         <v>2660.1372000000001</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16">
+        <v>80</v>
+      </c>
+      <c r="D16">
+        <v>80</v>
+      </c>
+      <c r="E16" t="str" cm="1">
+        <f t="array" ref="E16">_xlfn.IFS(ISBLANK(D16), "", D16 &lt;= 80, "0-80 days", D16 &lt;= 200, "81-200 days", D16 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>0-80 days</v>
+      </c>
+      <c r="F16">
+        <f>VLOOKUP(E16, $S$5:$V$7, 2, FALSE)</f>
+        <v>10.4</v>
+      </c>
+      <c r="G16">
+        <f>VLOOKUP(E16, $S$5:$V$7, 3, FALSE)</f>
+        <v>22</v>
+      </c>
+      <c r="H16">
+        <f>VLOOKUP(E16, $S$5:$V$7, 4, FALSE)</f>
+        <v>4.8</v>
+      </c>
+      <c r="I16">
+        <f>(5.11*F16 - 4*H16/100+2.26*G16/100)*10^-3</f>
+        <v>5.3449200000000009E-2</v>
+      </c>
+      <c r="J16">
+        <f>D16*I16*C16</f>
+        <v>342.07488000000006</v>
+      </c>
+      <c r="K16">
+        <f>$Q$4</f>
+        <v>28</v>
+      </c>
+      <c r="M16">
+        <f>SUM(J16:J18)</f>
+        <v>2412.0212615999999</v>
+      </c>
+      <c r="N16">
+        <f>M16*K16*10 ^ -3</f>
+        <v>67.536595324800004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B17" t="s">
+        <v>2</v>
+      </c>
+      <c r="C17">
+        <v>81</v>
+      </c>
+      <c r="D17">
+        <v>81</v>
+      </c>
+      <c r="E17" t="str" cm="1">
+        <f t="array" ref="E17">_xlfn.IFS(ISBLANK(D17), "", D17 &lt;= 80, "0-80 days", D17 &lt;= 200, "81-200 days", D17 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>81-200 days</v>
+      </c>
+      <c r="F17">
+        <f t="shared" ref="F17:F18" si="5">VLOOKUP(E17, $S$5:$V$7, 2, FALSE)</f>
+        <v>10.8</v>
+      </c>
+      <c r="G17">
+        <f t="shared" ref="G17:G18" si="6">VLOOKUP(E17, $S$5:$V$7, 3, FALSE)</f>
+        <v>22</v>
+      </c>
+      <c r="H17">
+        <f t="shared" ref="H17:H18" si="7">VLOOKUP(E17, $S$5:$V$7, 4, FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="I17">
+        <f t="shared" ref="I17:I18" si="8">(5.11*F17 - 4*H17/100+2.26*G17/100)*10^-3</f>
+        <v>5.5485200000000005E-2</v>
+      </c>
+      <c r="J17">
+        <f t="shared" ref="J17:J18" si="9">D17*I17*C17</f>
+        <v>364.03839720000008</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18">
+        <v>201</v>
+      </c>
+      <c r="D18">
+        <v>201</v>
+      </c>
+      <c r="E18" t="str" cm="1">
+        <f t="array" ref="E18">_xlfn.IFS(ISBLANK(D18), "", D18 &lt;= 80, "0-80 days", D18 &lt;= 200, "81-200 days", D18 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>201+ days</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="5"/>
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="6"/>
+        <v>24</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="7"/>
+        <v>5.5</v>
+      </c>
+      <c r="I18">
+        <f t="shared" si="8"/>
+        <v>4.2224400000000002E-2</v>
+      </c>
+      <c r="J18">
+        <f t="shared" si="9"/>
+        <v>1705.9079844</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>38</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+      <c r="D21">
+        <v>80</v>
+      </c>
+      <c r="E21" t="str" cm="1">
+        <f t="array" ref="E21">_xlfn.IFS(ISBLANK(D21), "", D21 &lt;= 80, "0-80 days", D21 &lt;= 200, "81-200 days", D21 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>0-80 days</v>
+      </c>
+      <c r="F21">
+        <f>VLOOKUP(E21, $S$5:$V$7, 2, FALSE)</f>
+        <v>10.4</v>
+      </c>
+      <c r="G21">
+        <f>VLOOKUP(E21, $S$5:$V$7, 3, FALSE)</f>
+        <v>22</v>
+      </c>
+      <c r="H21">
+        <f>VLOOKUP(E21, $S$5:$V$7, 4, FALSE)</f>
+        <v>4.8</v>
+      </c>
+      <c r="I21">
+        <f>(5.11*F21 - 4*H21/100+2.26*G21/100)*10^-3</f>
+        <v>5.3449200000000009E-2</v>
+      </c>
+      <c r="J21">
+        <f>D21*I21*C21</f>
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <f>$Q$4</f>
+        <v>28</v>
+      </c>
+      <c r="M21">
+        <f>SUM(J21:J23)</f>
+        <v>0</v>
+      </c>
+      <c r="N21">
+        <f>M21*K21*10 ^ -3</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+      <c r="D22">
+        <v>81</v>
+      </c>
+      <c r="E22" t="str" cm="1">
+        <f t="array" ref="E22">_xlfn.IFS(ISBLANK(D22), "", D22 &lt;= 80, "0-80 days", D22 &lt;= 200, "81-200 days", D22 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>81-200 days</v>
+      </c>
+      <c r="F22">
+        <f t="shared" ref="F22:F23" si="10">VLOOKUP(E22, $S$5:$V$7, 2, FALSE)</f>
+        <v>10.8</v>
+      </c>
+      <c r="G22">
+        <f t="shared" ref="G22:G23" si="11">VLOOKUP(E22, $S$5:$V$7, 3, FALSE)</f>
+        <v>22</v>
+      </c>
+      <c r="H22">
+        <f t="shared" ref="H22:H23" si="12">VLOOKUP(E22, $S$5:$V$7, 4, FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="I22">
+        <f t="shared" ref="I22:I23" si="13">(5.11*F22 - 4*H22/100+2.26*G22/100)*10^-3</f>
+        <v>5.5485200000000005E-2</v>
+      </c>
+      <c r="J22">
+        <f t="shared" ref="J22:J23" si="14">D22*I22*C22</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>201</v>
+      </c>
+      <c r="E23" t="str" cm="1">
+        <f t="array" ref="E23">_xlfn.IFS(ISBLANK(D23), "", D23 &lt;= 80, "0-80 days", D23 &lt;= 200, "81-200 days", D23 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>201+ days</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="10"/>
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="11"/>
+        <v>24</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="12"/>
+        <v>5.5</v>
+      </c>
+      <c r="I23">
+        <f t="shared" si="13"/>
+        <v>4.2224400000000002E-2</v>
+      </c>
+      <c r="J23">
+        <f t="shared" si="14"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>36</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1</v>
+      </c>
+      <c r="C31">
+        <v>100</v>
+      </c>
+      <c r="D31">
+        <v>70</v>
+      </c>
+      <c r="E31" t="str" cm="1">
+        <f t="array" ref="E31">_xlfn.IFS(ISBLANK(D31), "", D31 &lt;= 80, "0-80 days", D31 &lt;= 200, "81-200 days", D31 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>0-80 days</v>
+      </c>
+      <c r="F31">
+        <v>11</v>
+      </c>
+      <c r="G31">
+        <v>20</v>
+      </c>
+      <c r="H31">
+        <f>VLOOKUP(E31, $S$5:$V$7, 4, FALSE)</f>
+        <v>4.8</v>
+      </c>
+      <c r="I31">
+        <f>(5.11*F31 - 4*H31/100+2.26*G31/100)*10^-3</f>
+        <v>5.6469999999999999E-2</v>
+      </c>
+      <c r="J31">
+        <f>D31*I31*C31</f>
+        <v>395.29</v>
+      </c>
+      <c r="K31">
+        <f>$Q$4</f>
+        <v>28</v>
+      </c>
+      <c r="M31">
+        <f>SUM(J31:J33)</f>
+        <v>4420.2502000000004</v>
+      </c>
+      <c r="N31">
+        <f>M31*K31*10 ^ -3</f>
+        <v>123.7670056</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="B32" t="s">
+        <v>2</v>
+      </c>
+      <c r="C32">
+        <v>200</v>
+      </c>
+      <c r="D32">
+        <v>90</v>
+      </c>
+      <c r="E32" t="str" cm="1">
+        <f t="array" ref="E32">_xlfn.IFS(ISBLANK(D32), "", D32 &lt;= 80, "0-80 days", D32 &lt;= 200, "81-200 days", D32 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>81-200 days</v>
+      </c>
+      <c r="F32">
+        <v>12</v>
+      </c>
+      <c r="G32">
+        <v>21</v>
+      </c>
+      <c r="H32">
+        <f t="shared" ref="H32:H33" si="15">VLOOKUP(E32, $S$5:$V$7, 4, FALSE)</f>
+        <v>5</v>
+      </c>
+      <c r="I32">
+        <f t="shared" ref="I32:I33" si="16">(5.11*F32 - 4*H32/100+2.26*G32/100)*10^-3</f>
+        <v>6.1594600000000006E-2</v>
+      </c>
+      <c r="J32">
+        <f t="shared" ref="J32:J33" si="17">D32*I32*C32</f>
+        <v>1108.7028000000003</v>
+      </c>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B33" t="s">
+        <v>3</v>
+      </c>
+      <c r="C33">
+        <v>300</v>
+      </c>
+      <c r="D33">
+        <v>210</v>
+      </c>
+      <c r="E33" t="str" cm="1">
+        <f t="array" ref="E33">_xlfn.IFS(ISBLANK(D33), "", D33 &lt;= 80, "0-80 days", D33 &lt;= 200, "81-200 days", D33 &gt; 200, "201+ days", TRUE, "")</f>
+        <v>201+ days</v>
+      </c>
+      <c r="F33">
+        <v>9</v>
+      </c>
+      <c r="G33">
+        <v>23</v>
+      </c>
+      <c r="H33">
+        <f t="shared" si="15"/>
+        <v>5.5</v>
+      </c>
+      <c r="I33">
+        <f t="shared" si="16"/>
+        <v>4.6289799999999999E-2</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="17"/>
+        <v>2916.2574</v>
       </c>
     </row>
   </sheetData>

</xml_diff>